<commit_message>
CAR Varones: registro de limpieza sobre colector de 0.60 (abertura 0.70 apoyada en los muros) y DP-06D
- DP-06B y modelo 3D parametrizados por el ancho del colector (COLECTOR_B); Refugio sin cambios de geometria
- Varones: borde engrosado solo en 2 lados (1.20 m por registro), anclajes de los lados largos dentro del muro,
  barras transversales de borde con ganchos de 0.29 (L = 1.40)
- Planilla Varones: concreto del colector 56.02 -> 55.72 m3 (COLECTOR PARAMETROS C40 = 2 x b)
- DD-01, DA-02, especificaciones, memoria y LEEME actualizados; DP-06D agregada al juego de Varones
- DA-02 (ambos proyectos): total de concreto y nombre Delphin del acabado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_varones/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CON_COLECTOR.xlsx
+++ b/entregables_varones/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CON_COLECTOR.xlsx
@@ -515,7 +515,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2474" uniqueCount="1332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2474" uniqueCount="1339">
   <si>
     <t xml:space="preserve">RESUMEN METRADOS DE DRENAJE PLUVIAL</t>
   </si>
@@ -4525,6 +4525,27 @@
   </si>
   <si>
     <t xml:space="preserve">DESAGREGADO LLORADEROS fila 64 (DL-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Borde engrosado de la abertura: perimetro (solo los 2 lados transversales, entre muros)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lamina DP-06B: 2 x b; b = 0.60 es menor que la abertura de 0.70, en los lados largos el asiento es la cabeza del muro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REGISTROS DE LIMPIEZA EN LA LOSA DEL COLECTOR - lamina DP-06B (borde engrosado 0.15 x 0.10 solo en los 2 lados transversales, entre muros: en los lados largos la abertura apoya en la cabeza de los muros; descuento de la abertura 0.70 x 0.70 en la losa superior)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registros RV-01 a RV-11: borde engrosado de la abertura (2 lados, entre muros)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DP-06B, DD-01: 2 x 0.60 m por registro, en los 11 registros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lamina DP-01 (ubicacion), DP-06B, DP-06D, DD-01 y DD-02 (detalle): contramarco L 1 1/2"x1 1/2"x1/8" anclado a la losa y a la cabeza de los muros, marco L 1 1/2"x1 1/2"x1/8" soldado a la tapa, tapa de concreto armado 0.68 x 0.68 x 0.08 con parrilla 3/8" @0.10 y asas; abertura de 0.70 x 0.70 sobre el colector de 0.60: en los lados largos apoya en la cabeza de los muros y el borde engrosado 0.15 x 0.10 va solo en los 2 lados transversales. El registro de la caja CL pertenece al expediente del Hogar de Refugio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bordes engrosados de abertura de registros RV-01 a RV-11 (2 lados, entre muros)</t>
   </si>
 </sst>
 </file>
@@ -7868,7 +7889,7 @@
       </c>
       <c r="D65" s="16" t="n">
         <f aca="false">+'PLANILLA GENERAL DE METRADOS'!K176</f>
-        <v>56.017129</v>
+        <v>55.720129</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12219,16 +12240,17 @@
         <v>31</v>
       </c>
       <c r="B40" s="150" t="s">
-        <v>588</v>
+        <v>1332</v>
       </c>
       <c r="C40" s="289" t="n">
-        <v>3</v>
+        <f aca="false">2*C10</f>
+        <v>1.2</v>
       </c>
       <c r="D40" s="290" t="s">
         <v>71</v>
       </c>
       <c r="E40" s="272" t="s">
-        <v>589</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13385,7 +13407,7 @@
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="296" t="s">
-        <v>649</v>
+        <v>1334</v>
       </c>
       <c r="B15" s="296"/>
       <c r="C15" s="296"/>
@@ -13450,14 +13472,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="150" t="s">
-        <v>657</v>
+        <v>1335</v>
       </c>
       <c r="C17" s="269" t="s">
         <v>658</v>
       </c>
       <c r="D17" s="271" t="n">
         <f aca="false">'COLECTOR PARAMETROS'!$C$40</f>
-        <v>3.0</v>
+        <v>1.2</v>
       </c>
       <c r="E17" s="271" t="n">
         <f aca="false">'COLECTOR PARAMETROS'!$C$41</f>
@@ -13475,12 +13497,12 @@
       <c r="J17" s="22"/>
       <c r="K17" s="271" t="n">
         <f aca="false">D17*E17*F17*G17</f>
-        <v>0.495</v>
+        <v>0.198</v>
       </c>
       <c r="L17" s="22"/>
       <c r="M17" s="22"/>
       <c r="N17" s="272" t="s">
-        <v>659</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13546,7 +13568,7 @@
       </c>
       <c r="K19" s="295" t="n">
         <f aca="false">SUM(K17:K18)</f>
-        <v>-0.0439999999999999</v>
+        <v>-0.341</v>
       </c>
       <c r="L19" s="295" t="n">
         <f aca="false">SUM(L17:L18)</f>
@@ -13673,11 +13695,11 @@
       </c>
       <c r="H25" s="271" t="n">
         <f aca="false">K19</f>
-        <v>-0.0439999999999999</v>
+        <v>-0.341</v>
       </c>
       <c r="I25" s="298" t="n">
         <f aca="false">G25+H25</f>
-        <v>10.2529</v>
+        <v>9.9559</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17711,7 +17733,7 @@
       <c r="J176" s="26"/>
       <c r="K176" s="26" t="n">
         <f aca="false">SUM(J177:J189)</f>
-        <v>56.017129</v>
+        <v>55.720129</v>
       </c>
       <c r="L176" s="25" t="s">
         <v>25</v>
@@ -17941,7 +17963,7 @@
     <row r="188" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="27"/>
       <c r="B188" s="27" t="s">
-        <v>201</v>
+        <v>1338</v>
       </c>
       <c r="C188" s="28" t="n">
         <v>1</v>
@@ -17954,7 +17976,7 @@
       <c r="I188" s="28"/>
       <c r="J188" s="28" t="n">
         <f aca="false">'COLECTOR CONCRETO'!K17</f>
-        <v>0.495</v>
+        <v>0.198</v>
       </c>
       <c r="K188" s="28"/>
       <c r="L188" s="27"/>
@@ -19986,7 +20008,7 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="267" t="s">
-        <v>876</v>
+        <v>1337</v>
       </c>
       <c r="B7" s="267"/>
       <c r="C7" s="267"/>
@@ -21328,7 +21350,7 @@
       </c>
       <c r="D28" s="271" t="n">
         <f aca="false">SUM('PLANILLA GENERAL DE METRADOS'!J185:J189)</f>
-        <v>10.2529</v>
+        <v>9.9559</v>
       </c>
       <c r="E28" s="297" t="s">
         <v>802</v>
@@ -21341,7 +21363,7 @@
       </c>
       <c r="H28" s="298" t="n">
         <f aca="false">G28*$D$28</f>
-        <v>99.760717</v>
+        <v>96.870907</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21360,7 +21382,7 @@
       </c>
       <c r="H29" s="298" t="n">
         <f aca="false">G29*$D$28</f>
-        <v>5.331508</v>
+        <v>5.177068</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21379,7 +21401,7 @@
       </c>
       <c r="H30" s="298" t="n">
         <f aca="false">G30*$D$28</f>
-        <v>5.434037</v>
+        <v>5.276627</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21398,7 +21420,7 @@
       </c>
       <c r="H31" s="298" t="n">
         <f aca="false">G31*$D$28</f>
-        <v>1.9070394</v>
+        <v>1.8517974</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21417,7 +21439,7 @@
       </c>
       <c r="H32" s="298" t="n">
         <f aca="false">G32*$D$28</f>
-        <v>8.20232</v>
+        <v>7.96472</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21436,7 +21458,7 @@
       </c>
       <c r="H33" s="298" t="n">
         <f aca="false">G33*$D$28</f>
-        <v>8.20232</v>
+        <v>7.96472</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21455,7 +21477,7 @@
       </c>
       <c r="H34" s="298" t="n">
         <f aca="false">G34*$D$28</f>
-        <v>8.20232</v>
+        <v>7.96472</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21474,7 +21496,7 @@
       </c>
       <c r="H35" s="298" t="n">
         <f aca="false">G35*$D$28</f>
-        <v>8.20232</v>
+        <v>7.96472</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21493,7 +21515,7 @@
       </c>
       <c r="H36" s="298" t="n">
         <f aca="false">G36*$D$28</f>
-        <v>65.61856</v>
+        <v>63.71776</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>